<commit_message>
All Pennik models working.
</commit_message>
<xml_diff>
--- a/Projects/Pennink-Model/cases/Boogkanaal1/Boogkanaal1.xlsx
+++ b/Projects/Pennink-Model/cases/Boogkanaal1/Boogkanaal1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Theo/GRWMODELS/python/mf6lab/Projects/Pennink-Model/cases/Boogkanaal1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11F13443-8AB7-D241-A5BD-8F3FDDF0E35D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0800BF6-848D-F142-ADFA-1EC8F097FE92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9820" yWindow="-24220" windowWidth="28180" windowHeight="16980" tabRatio="751" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3640" yWindow="2280" windowWidth="28180" windowHeight="16980" tabRatio="751" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NAM" sheetId="1" r:id="rId1"/>
@@ -126,7 +126,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2458" uniqueCount="424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2456" uniqueCount="424">
   <si>
     <t>ON / OFF</t>
   </si>
@@ -1397,7 +1397,7 @@
     <t>Days</t>
   </si>
   <si>
-    <t>COMPLEX</t>
+    <t>NEWTON</t>
   </si>
 </sst>
 </file>
@@ -3603,7 +3603,7 @@
         <v>108</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>423</v>
+        <v>379</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>380</v>
@@ -3682,8 +3682,8 @@
       <c r="B18" t="s">
         <v>115</v>
       </c>
-      <c r="C18" t="s">
-        <v>19</v>
+      <c r="C18">
+        <v>9.9999999999999995E-7</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.15">
@@ -3704,8 +3704,8 @@
       <c r="B20" t="s">
         <v>117</v>
       </c>
-      <c r="C20" t="s">
-        <v>19</v>
+      <c r="C20">
+        <v>800</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.15">
@@ -5762,7 +5762,7 @@
         <v>43</v>
       </c>
       <c r="C218" s="9" t="s">
-        <v>382</v>
+        <v>423</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.15">

</xml_diff>